<commit_message>
Revisions to Syllabus 2026 and W1S1 content.
</commit_message>
<xml_diff>
--- a/Syllabus/Weeks_Table.xlsx
+++ b/Syllabus/Weeks_Table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sutdapac-my.sharepoint.com/personal/matthieu_demari_sutd_edu_sg/Documents/Teaching folder for web/9. DL @ SUTD 2021-ongoing/Teaching Materials/1. Lectures/Syllabus/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sutdapac-my.sharepoint.com/personal/matthieu_demari_sutd_edu_sg/Documents/Teaching folder for web/50.039 DL/Teaching Materials/1. Lectures/Syllabus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="174" documentId="11_F25DC773A252ABDACC10480EB1D941EE5BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9815AEE9-0728-4EC2-8497-88819F2D7C61}"/>
+  <xr:revisionPtr revIDLastSave="177" documentId="11_F25DC773A252ABDACC10480EB1D941EE5BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F652347-7685-4938-8C99-521BAA23ED5C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-60" yWindow="14292" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -205,7 +205,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -242,12 +242,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="16">
     <border>
@@ -458,11 +452,38 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -472,25 +493,22 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -509,39 +527,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -834,317 +819,329 @@
   <sheetData>
     <row r="1" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B3" s="6">
+      <c r="B3" s="9">
         <v>1</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="4"/>
-    </row>
-    <row r="4" spans="2:5" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="7"/>
-      <c r="C4" s="9" t="s">
+      <c r="D3" s="12"/>
+      <c r="E3" s="13"/>
+    </row>
+    <row r="4" spans="2:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="10"/>
+      <c r="C4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="27" t="s">
+      <c r="E4" s="4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B5" s="6">
+      <c r="B5" s="9">
         <v>2</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="4"/>
-    </row>
-    <row r="6" spans="2:5" ht="135.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="7"/>
-      <c r="C6" s="9" t="s">
+      <c r="D5" s="12"/>
+      <c r="E5" s="13"/>
+    </row>
+    <row r="6" spans="2:5" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="10"/>
+      <c r="C6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B7" s="6">
+      <c r="B7" s="9">
         <v>3</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="3"/>
-      <c r="E7" s="4"/>
-    </row>
-    <row r="8" spans="2:5" ht="135.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="7"/>
-      <c r="C8" s="9" t="s">
+      <c r="D7" s="12"/>
+      <c r="E7" s="13"/>
+    </row>
+    <row r="8" spans="2:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="10"/>
+      <c r="C8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="6" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B9" s="6">
+      <c r="B9" s="9">
         <v>4</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="3"/>
-      <c r="E9" s="4"/>
-    </row>
-    <row r="10" spans="2:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="7"/>
-      <c r="C10" s="9" t="s">
+      <c r="D9" s="12"/>
+      <c r="E9" s="13"/>
+    </row>
+    <row r="10" spans="2:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="10"/>
+      <c r="C10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" s="6" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B11" s="6">
+      <c r="B11" s="9">
         <v>5</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="3"/>
-      <c r="E11" s="4"/>
-    </row>
-    <row r="12" spans="2:5" ht="135.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="7"/>
-      <c r="C12" s="9" t="s">
+      <c r="D11" s="12"/>
+      <c r="E11" s="13"/>
+    </row>
+    <row r="12" spans="2:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="10"/>
+      <c r="C12" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="6" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B13" s="6">
+      <c r="B13" s="9">
         <v>6</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="3"/>
-      <c r="E13" s="4"/>
-    </row>
-    <row r="14" spans="2:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="7"/>
-      <c r="C14" s="9" t="s">
+      <c r="D13" s="12"/>
+      <c r="E13" s="13"/>
+    </row>
+    <row r="14" spans="2:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="10"/>
+      <c r="C14" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E14" s="11" t="s">
+      <c r="E14" s="6" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B15" s="6">
+      <c r="B15" s="9">
         <v>7</v>
       </c>
-      <c r="C15" s="20" t="s">
+      <c r="C15" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="21"/>
-      <c r="E15" s="22"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="16"/>
     </row>
     <row r="16" spans="2:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="7"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="25"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="19"/>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B17" s="6">
+      <c r="B17" s="9">
         <v>8</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="3"/>
-      <c r="E17" s="4"/>
-    </row>
-    <row r="18" spans="2:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="7"/>
-      <c r="C18" s="9" t="s">
+      <c r="D17" s="12"/>
+      <c r="E17" s="13"/>
+    </row>
+    <row r="18" spans="2:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="10"/>
+      <c r="C18" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E18" s="11" t="s">
+      <c r="E18" s="6" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B19" s="6">
+      <c r="B19" s="9">
         <v>9</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="D19" s="3"/>
-      <c r="E19" s="4"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="13"/>
     </row>
     <row r="20" spans="2:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="7"/>
-      <c r="C20" s="9" t="s">
+      <c r="B20" s="10"/>
+      <c r="C20" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="E20" s="6" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B21" s="6">
+      <c r="B21" s="9">
         <v>10</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="D21" s="3"/>
-      <c r="E21" s="4"/>
-    </row>
-    <row r="22" spans="2:5" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="7"/>
-      <c r="C22" s="28" t="s">
+      <c r="D21" s="12"/>
+      <c r="E21" s="13"/>
+    </row>
+    <row r="22" spans="2:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="10"/>
+      <c r="C22" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E22" s="11" t="s">
+      <c r="E22" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B23" s="6">
+      <c r="B23" s="9">
         <v>11</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="D23" s="3"/>
-      <c r="E23" s="4"/>
-    </row>
-    <row r="24" spans="2:5" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="7"/>
-      <c r="C24" s="9" t="s">
+      <c r="D23" s="12"/>
+      <c r="E23" s="13"/>
+    </row>
+    <row r="24" spans="2:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="10"/>
+      <c r="C24" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E24" s="11" t="s">
+      <c r="E24" s="6" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B25" s="6">
+      <c r="B25" s="9">
         <v>12</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="D25" s="3"/>
-      <c r="E25" s="4"/>
-    </row>
-    <row r="26" spans="2:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="7"/>
-      <c r="C26" s="9" t="s">
+      <c r="D25" s="12"/>
+      <c r="E25" s="13"/>
+    </row>
+    <row r="26" spans="2:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="10"/>
+      <c r="C26" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E26" s="11" t="s">
+      <c r="E26" s="6" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B27" s="6">
+      <c r="B27" s="9">
         <v>13</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="D27" s="3"/>
-      <c r="E27" s="4"/>
-    </row>
-    <row r="28" spans="2:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="7"/>
-      <c r="C28" s="18" t="s">
+      <c r="D27" s="12"/>
+      <c r="E27" s="13"/>
+    </row>
+    <row r="28" spans="2:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="10"/>
+      <c r="C28" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="D28" s="19" t="s">
+      <c r="D28" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="E28" s="11" t="s">
+      <c r="E28" s="6" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B29" s="6">
+      <c r="B29" s="9">
         <v>14</v>
       </c>
-      <c r="C29" s="12" t="s">
+      <c r="C29" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="D29" s="13"/>
-      <c r="E29" s="14"/>
+      <c r="D29" s="21"/>
+      <c r="E29" s="22"/>
     </row>
     <row r="30" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="7"/>
-      <c r="C30" s="15"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="17"/>
+      <c r="B30" s="10"/>
+      <c r="C30" s="23"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:E13"/>
     <mergeCell ref="B27:B28"/>
     <mergeCell ref="C27:E27"/>
     <mergeCell ref="B29:B30"/>
@@ -1161,18 +1158,6 @@
     <mergeCell ref="C17:E17"/>
     <mergeCell ref="B19:B20"/>
     <mergeCell ref="C19:E19"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:E7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>